<commit_message>
chore: add work assignment backend, scripts, docs, and analysis files
</commit_message>
<xml_diff>
--- a/docs/kadavanthra&EDAPPALLY fee structure newww.xlsx
+++ b/docs/kadavanthra&EDAPPALLY fee structure newww.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjun\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22C221D-7AA0-4C33-B691-9EC0E8FDB18C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D8FA1F-8D38-4638-94C2-12017A0025B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{72A80A32-F8D7-40E2-A7D1-6AA8071C64B1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{72A80A32-F8D7-40E2-A7D1-6AA8071C64B1}"/>
   </bookViews>
   <sheets>
     <sheet name="KADAVANTHARA" sheetId="1" r:id="rId1"/>
@@ -26,10 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="33">
-  <si>
-    <t>Basic Fees Structure - Kadavanthra Branch</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="34">
   <si>
     <t>Class</t>
   </si>
@@ -116,9 +113,6 @@
     <t>10th-subject wise</t>
   </si>
   <si>
-    <t>Basic Fees Structure - Edappally Branch</t>
-  </si>
-  <si>
     <t>9 State</t>
   </si>
   <si>
@@ -126,6 +120,15 @@
   </si>
   <si>
     <t xml:space="preserve">Plus One </t>
+  </si>
+  <si>
+    <t>Advanced Fees Structure - Edappally Branch</t>
+  </si>
+  <si>
+    <t>Advanced Fees Structure - Kadavanthra Branch</t>
+  </si>
+  <si>
+    <t>Advanced  Fees Structure - Kadavanthra Branch</t>
   </si>
 </sst>
 </file>
@@ -302,12 +305,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -315,6 +312,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -638,50 +641,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="A1" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
     </row>
     <row r="2" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>34500</v>
@@ -696,21 +699,21 @@
         <v>29500</v>
       </c>
       <c r="F3" s="2">
-        <v>8300</v>
+        <v>10300</v>
       </c>
       <c r="G3" s="2">
-        <v>6000</v>
+        <v>7400</v>
       </c>
       <c r="H3" s="2">
-        <v>6000</v>
+        <v>7400</v>
       </c>
       <c r="I3" s="2">
-        <v>3500</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="2">
         <v>27800</v>
@@ -739,7 +742,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="2">
         <v>34500</v>
@@ -768,7 +771,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2">
         <v>41100</v>
@@ -797,7 +800,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="2">
         <v>41100</v>
@@ -847,50 +850,50 @@
       <c r="I9" s="3"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
+      <c r="A10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>2</v>
-      </c>
       <c r="C11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="G11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="I11" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2">
         <v>34500</v>
@@ -919,7 +922,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2">
         <v>34500</v>
@@ -948,7 +951,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2">
         <v>41100</v>
@@ -977,7 +980,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2">
         <v>41100</v>
@@ -1005,50 +1008,50 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+      <c r="A18" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
     </row>
     <row r="19" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="2">
         <v>16700</v>
@@ -1077,7 +1080,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="2">
         <v>16700</v>
@@ -1106,7 +1109,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="2">
         <v>16700</v>
@@ -1156,50 +1159,50 @@
       <c r="I24" s="3"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
+      <c r="A25" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="13"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
     </row>
     <row r="26" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="F26" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="G26" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="H26" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="I26" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" s="2">
         <v>16700</v>
@@ -1228,7 +1231,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B28" s="2">
         <v>16700</v>
@@ -1257,7 +1260,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B29" s="2">
         <v>16700</v>
@@ -1285,50 +1288,50 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
+      <c r="A32" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
     </row>
     <row r="33" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="G33" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="H33" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="I33" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B34" s="2">
         <v>9400</v>
@@ -1357,7 +1360,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B35" s="2">
         <v>9400</v>
@@ -1386,7 +1389,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B36" s="2">
         <v>9400</v>
@@ -1415,7 +1418,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B37" s="2">
         <v>15600</v>
@@ -1444,50 +1447,50 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="16"/>
+      <c r="A39" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="13"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="14"/>
     </row>
     <row r="40" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="F40" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="G40" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="I40" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="I40" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B41" s="2">
         <v>9400</v>
@@ -1516,7 +1519,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B42" s="2">
         <v>9400</v>
@@ -1545,7 +1548,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B43" s="2">
         <v>9400</v>
@@ -1574,7 +1577,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B44" s="2">
         <v>15600</v>
@@ -1616,54 +1619,54 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2138A6F0-DF16-48F4-AA8C-B0829BB91FF8}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="A1" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
     </row>
     <row r="2" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B3" s="2">
         <v>27800</v>
@@ -1692,7 +1695,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2">
         <v>34500</v>
@@ -1721,7 +1724,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2">
         <v>27800</v>
@@ -1750,7 +1753,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2">
         <v>34500</v>
@@ -1779,7 +1782,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2">
         <v>41100</v>
@@ -1808,7 +1811,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2">
         <v>41100</v>
@@ -1847,50 +1850,50 @@
       <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
+      <c r="A10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>2</v>
-      </c>
       <c r="C11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="G11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="I11" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B12" s="9">
         <v>27800</v>
@@ -1919,7 +1922,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="2">
         <v>34500</v>
@@ -1948,7 +1951,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B14" s="9">
         <v>27800</v>
@@ -1977,7 +1980,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="2">
         <v>34500</v>
@@ -2006,7 +2009,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="2">
         <v>41100</v>
@@ -2035,7 +2038,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="2">
         <v>41100</v>
@@ -2062,611 +2065,10 @@
         <v>4100</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-    </row>
-    <row r="24" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="2">
-        <v>16700</v>
-      </c>
-      <c r="C25" s="2">
-        <v>15000</v>
-      </c>
-      <c r="D25" s="2">
-        <v>13800</v>
-      </c>
-      <c r="E25" s="2">
-        <v>14200</v>
-      </c>
-      <c r="F25" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G25" s="2">
-        <v>3500</v>
-      </c>
-      <c r="H25" s="2">
-        <v>3500</v>
-      </c>
-      <c r="I25" s="2">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="2">
-        <v>16700</v>
-      </c>
-      <c r="C26" s="2">
-        <v>15000</v>
-      </c>
-      <c r="D26" s="2">
-        <v>13800</v>
-      </c>
-      <c r="E26" s="2">
-        <v>14200</v>
-      </c>
-      <c r="F26" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G26" s="2">
-        <v>3500</v>
-      </c>
-      <c r="H26" s="2">
-        <v>3500</v>
-      </c>
-      <c r="I26" s="2">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="2">
-        <v>16700</v>
-      </c>
-      <c r="C27" s="2">
-        <v>15000</v>
-      </c>
-      <c r="D27" s="2">
-        <v>13800</v>
-      </c>
-      <c r="E27" s="2">
-        <v>14200</v>
-      </c>
-      <c r="F27" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G27" s="2">
-        <v>3500</v>
-      </c>
-      <c r="H27" s="2">
-        <v>3500</v>
-      </c>
-      <c r="I27" s="2">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-    </row>
-    <row r="31" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H31" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B32" s="2">
-        <v>16700</v>
-      </c>
-      <c r="C32" s="2">
-        <v>15000</v>
-      </c>
-      <c r="D32" s="7">
-        <v>14600</v>
-      </c>
-      <c r="E32" s="7">
-        <v>2500</v>
-      </c>
-      <c r="F32" s="7">
-        <v>2100</v>
-      </c>
-      <c r="G32" s="2">
-        <v>15000</v>
-      </c>
-      <c r="H32" s="8">
-        <v>1900</v>
-      </c>
-      <c r="I32" s="8">
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" s="2">
-        <v>16700</v>
-      </c>
-      <c r="C33" s="2">
-        <v>15000</v>
-      </c>
-      <c r="D33" s="7">
-        <v>14600</v>
-      </c>
-      <c r="E33" s="7">
-        <v>2500</v>
-      </c>
-      <c r="F33" s="7">
-        <v>2100</v>
-      </c>
-      <c r="G33" s="2">
-        <v>15000</v>
-      </c>
-      <c r="H33" s="8">
-        <v>1900</v>
-      </c>
-      <c r="I33" s="8">
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B34" s="2">
-        <v>16700</v>
-      </c>
-      <c r="C34" s="2">
-        <v>15000</v>
-      </c>
-      <c r="D34" s="7">
-        <v>14600</v>
-      </c>
-      <c r="E34" s="7">
-        <v>2500</v>
-      </c>
-      <c r="F34" s="7">
-        <v>2100</v>
-      </c>
-      <c r="G34" s="2">
-        <v>15000</v>
-      </c>
-      <c r="H34" s="8">
-        <v>1900</v>
-      </c>
-      <c r="I34" s="8">
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
-    </row>
-    <row r="38" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I38" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B39" s="2">
-        <v>9400</v>
-      </c>
-      <c r="C39" s="2">
-        <v>8500</v>
-      </c>
-      <c r="D39" s="2">
-        <v>7900</v>
-      </c>
-      <c r="E39" s="2">
-        <v>8100</v>
-      </c>
-      <c r="F39" s="2">
-        <v>2800</v>
-      </c>
-      <c r="G39" s="2">
-        <v>2000</v>
-      </c>
-      <c r="H39" s="2">
-        <v>2000</v>
-      </c>
-      <c r="I39" s="2">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B40" s="2">
-        <v>9400</v>
-      </c>
-      <c r="C40" s="2">
-        <v>8500</v>
-      </c>
-      <c r="D40" s="2">
-        <v>7900</v>
-      </c>
-      <c r="E40" s="2">
-        <v>8100</v>
-      </c>
-      <c r="F40" s="2">
-        <v>2800</v>
-      </c>
-      <c r="G40" s="2">
-        <v>2000</v>
-      </c>
-      <c r="H40" s="2">
-        <v>2000</v>
-      </c>
-      <c r="I40" s="2">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B41" s="2">
-        <v>9400</v>
-      </c>
-      <c r="C41" s="2">
-        <v>8500</v>
-      </c>
-      <c r="D41" s="2">
-        <v>7900</v>
-      </c>
-      <c r="E41" s="2">
-        <v>8100</v>
-      </c>
-      <c r="F41" s="2">
-        <v>2800</v>
-      </c>
-      <c r="G41" s="2">
-        <v>2000</v>
-      </c>
-      <c r="H41" s="2">
-        <v>2000</v>
-      </c>
-      <c r="I41" s="2">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B42" s="2">
-        <v>15600</v>
-      </c>
-      <c r="C42" s="2">
-        <v>14000</v>
-      </c>
-      <c r="D42" s="2">
-        <v>12900</v>
-      </c>
-      <c r="E42" s="2">
-        <f>C42*95%</f>
-        <v>13300</v>
-      </c>
-      <c r="F42" s="2">
-        <v>4700</v>
-      </c>
-      <c r="G42" s="2">
-        <v>3300</v>
-      </c>
-      <c r="H42" s="2">
-        <v>3300</v>
-      </c>
-      <c r="I42" s="2">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B44" s="15"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
-      <c r="G44" s="16"/>
-      <c r="H44" s="16"/>
-      <c r="I44" s="16"/>
-    </row>
-    <row r="45" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I45" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B46" s="2">
-        <v>9400</v>
-      </c>
-      <c r="C46" s="2">
-        <v>8500</v>
-      </c>
-      <c r="D46" s="7">
-        <v>8300</v>
-      </c>
-      <c r="E46" s="7">
-        <v>1400</v>
-      </c>
-      <c r="F46" s="7">
-        <v>1300</v>
-      </c>
-      <c r="G46" s="2">
-        <v>8500</v>
-      </c>
-      <c r="H46" s="8">
-        <v>1100</v>
-      </c>
-      <c r="I46" s="8">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B47" s="2">
-        <v>9400</v>
-      </c>
-      <c r="C47" s="2">
-        <v>8500</v>
-      </c>
-      <c r="D47" s="7">
-        <v>8300</v>
-      </c>
-      <c r="E47" s="7">
-        <v>1400</v>
-      </c>
-      <c r="F47" s="7">
-        <v>1300</v>
-      </c>
-      <c r="G47" s="2">
-        <v>8500</v>
-      </c>
-      <c r="H47" s="8">
-        <v>1100</v>
-      </c>
-      <c r="I47" s="8">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B48" s="2">
-        <v>9400</v>
-      </c>
-      <c r="C48" s="2">
-        <v>8500</v>
-      </c>
-      <c r="D48" s="7">
-        <v>8300</v>
-      </c>
-      <c r="E48" s="7">
-        <v>1400</v>
-      </c>
-      <c r="F48" s="7">
-        <v>1300</v>
-      </c>
-      <c r="G48" s="2">
-        <v>8500</v>
-      </c>
-      <c r="H48" s="8">
-        <v>1100</v>
-      </c>
-      <c r="I48" s="8">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B49" s="2">
-        <v>15600</v>
-      </c>
-      <c r="C49" s="2">
-        <v>14000</v>
-      </c>
-      <c r="D49" s="7">
-        <v>13600</v>
-      </c>
-      <c r="E49" s="7">
-        <v>2300</v>
-      </c>
-      <c r="F49" s="7">
-        <v>2100</v>
-      </c>
-      <c r="G49" s="2">
-        <v>14000</v>
-      </c>
-      <c r="H49" s="8">
-        <v>1800</v>
-      </c>
-      <c r="I49" s="8">
-        <v>1400</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A44:I44"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A37:I37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>